<commit_message>
ADNOCLS: deliverables rebuilt on the sanctioned beta and published to files/
The rebuild agent died mid-edit on a server error, leaving three gate scripts
referencing a lead-lag sum beta the model no longer produces -- the sanctioned
routine returns a Blume shrink instead. All three now check the figure the model
actually publishes, and the workbook gates pass again.

Study 52 pages, bibliography 37, workbook 130. The copies under files/ now carry
the same beta, cost of capital and central as the page that links to them; the
one remaining mention of the old slope is the sentence that explains the change.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FX6uP9o59mB1WpgL9CePqV
</commit_message>
<xml_diff>
--- a/files/ADNOCLS_Valuation_Model_09082026.xlsx
+++ b/files/ADNOCLS_Valuation_Model_09082026.xlsx
@@ -545,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I115"/>
+  <dimension ref="A1:I126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="114" customWidth="1" min="1" max="1"/>
@@ -970,352 +970,425 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>How revenue is built. Not as one growth rate, and not off the published rate either. The company gives one</t>
+          <t>AND THE BETA HAS BEEN RE-MEASURED. It is now produced by the same standard routine used for every share</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>rate per vessel class each quarter, and its own chief financial officer said on the first-quarter call that</t>
+          <t>covered on this desk: the market series is resolved from the exchange the share is listed on rather than</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>this rate is a BLEND across the whole class, the vessels on charters out included. So the SPOT rate is not</t>
+          <t>chosen, both series are screened for data quality before they are paired, and the weekly returns are</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>read off that disclosure — it is SOLVED out of it, window by window: the published blend times the class</t>
+          <t>measured on that exchange's own trading week. The series it resolved is the one this study already used, so</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>vessel-days, less the revenue the twelve disclosed fixtures earn over exactly the days their own contracts</t>
+          <t>WHICH market the share is measured against has not changed — but the grid and the screening do move the</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>run, divided by the vessel-days that actually traded spot. Every step of that derivation is on the Segments</t>
+          <t>figure: the slope is now 1.1032 on 159 weekly observations, and its 90% confidence interval</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>sheet, cell by cell. The forecast then prices each vessel on its own terms — chartered vessels at their</t>
+          <t>runs 0.586 to 1.621, materially WIDER than the interval the previous edition</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>contracted rate for their contracted days, everything else at the implied spot rate — less an all-in running</t>
+          <t>published. The bear and bull cases take those two bounds directly, so the published range widens with it.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>cost per vessel-day that is itself solved so the same construction reproduces the tanker earnings the company</t>
+          <t>A range that widens on re-measurement is information about how much a three-year price history can settle,</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>reported for 2025. The gas carriers are contracted vessel-years times a day rate solved the same way. The</t>
+          <t>not an embarrassment to be smoothed away.</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>five remaining units are grown on their own revenue and margin drivers, anchored on what each actually</t>
-        </is>
-      </c>
+      <c r="A72" s="3" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>earned in the first quarter of 2026.</t>
+          <t>How revenue is built. Not as one growth rate, and not off the published rate either. The company gives one</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="3" t="inlineStr"/>
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>rate per vessel class each quarter, and its own chief financial officer said on the first-quarter call that</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>THE COST OF CAPITAL CARRIES THREE TRANCHES, NOT TWO: equity, debt, and the perpetual capital securities at</t>
+          <t>this rate is a BLEND across the whole class, the vessels on charters out included. So the SPOT rate is not</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>their own coupon. Those securities rank ahead of the ordinary shares and are deducted in the equity bridge,</t>
+          <t>read off that disclosure — it is SOLVED out of it, window by window: the published blend times the class</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>and a claim that is deducted from enterprise value has to be weighted in the rate as well — the two are</t>
+          <t>vessel-days, less the revenue the twelve disclosed fixtures earn over exactly the days their own contracts</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>halves of one treatment. The coupon is an equity distribution rather than interest, so it is not taxed down.</t>
+          <t>run, divided by the vessel-days that actually traded spot. Every step of that derivation is on the Segments</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>Every construction in the workbook carries the same three tranches, including the sensitivity re-runs, so</t>
+          <t>sheet, cell by cell. The forecast then prices each vessel on its own terms — chartered vessels at their</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>the sensitivity grid is centred on the figure it brackets.</t>
+          <t>contracted rate for their contracted days, everything else at the implied spot rate — less an all-in running</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="3" t="inlineStr"/>
+      <c r="A81" s="3" t="inlineStr">
+        <is>
+          <t>cost per vessel-day that is itself solved so the same construction reproduces the tanker earnings the company</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>THE BOOK LENS IS A RESIDUAL INCOME BUILD. A single-stage justified price-to-book assumes a steady state this</t>
+          <t>reported for 2025. The gas carriers are contracted vessel-years times a day rate solved the same way. The</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>company is not in: it pays out about a third of its earnings and compounds its book above its own cost of</t>
+          <t>five remaining units are grown on their own revenue and margin drivers, anchored on what each actually</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>equity, where that formula is undefined rather than merely wrong. The lens is instead the book the company</t>
+          <t>earned in the first quarter of 2026.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="3" t="inlineStr">
-        <is>
-          <t>already has, plus the present value of earning more than the cost of equity on it for five years, plus a</t>
-        </is>
-      </c>
+      <c r="A85" s="3" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>remainder in which that excess fades. The whole ladder is live on the Relative &amp; Normalized sheet, three</t>
+          <t>THE COST OF CAPITAL CARRIES THREE TRANCHES, NOT TWO: equity, debt, and the perpetual capital securities at</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>times over — base, bear and bull — and the return it is struck on is what the ORDINARY holders earn, after</t>
+          <t>their own coupon. Those securities rank ahead of the ordinary shares and are deducted in the equity bridge,</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>the perpetual coupon that ranks ahead of them.</t>
+          <t>and a claim that is deducted from enterprise value has to be weighted in the rate as well — the two are</t>
         </is>
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="3" t="inlineStr"/>
+      <c r="A89" s="3" t="inlineStr">
+        <is>
+          <t>halves of one treatment. The coupon is an equity distribution rather than interest, so it is not taxed down.</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>THE CONTESTED JUDGEMENT, PUBLISHED BOTH WAYS — HOW THE MARKET IS MEASURED. The same weekly regression of the</t>
+          <t>Every construction in the workbook carries the same three tranches, including the sensitivity re-runs, so</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>stock's own returns is run against two different measures of its market, and the answer moves a long way</t>
+          <t>the sensitivity grid is centred on the figure it brackets.</t>
         </is>
       </c>
     </row>
     <row r="92">
-      <c r="A92" s="3" t="inlineStr">
-        <is>
-          <t>between them. Against the published index of the exchange the share is listed on — the index the method</t>
-        </is>
-      </c>
+      <c r="A92" s="3" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>asks for, and the primary reading — the beta is 1.085. Against an equal-weight composite of that same</t>
+          <t>THE BOOK LENS IS A RESIDUAL INCOME BUILD. A single-stage justified price-to-book assumes a steady state this</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>exchange's names, which gives its smallest listings the same say as its largest, the beta is</t>
+          <t>company is not in: it pays out about a third of its earnings and compounds its book above its own cost of</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>0.705. The published index is weighted by size and is therefore dominated by the very group this</t>
+          <t>equity, where that formula is undefined rather than merely wrong. The lens is instead the book the company</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>company belongs to; the composite is not. That single difference in construction, and nothing about the</t>
+          <t>already has, plus the present value of earning more than the cost of equity on it for five years, plus a</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>company, moves the cost of equity and the cash-flow value materially. BOTH are carried through the model in</t>
+          <t>remainder in which that excess fades. The whole ladder is live on the Relative &amp; Normalized sheet, three</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>full, side by side, on the Summary, Fundamental Valuation and DCF sheets. They are NOT averaged into one</t>
+          <t>times over — base, bear and bull — and the return it is struck on is what the ORDINARY holders earn, after</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>number. The regression's own 90% confidence interval on the primary estimate runs 0.758 to 1.412, and</t>
+          <t>the perpetual coupon that ranks ahead of them.</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="3" t="inlineStr">
-        <is>
-          <t>those two bounds — not round numbers chosen by hand — are the betas used in the bear and bull cases, so the</t>
-        </is>
-      </c>
+      <c r="A100" s="3" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>published range is the range the estimate itself supports.</t>
+          <t>THE CONTESTED JUDGEMENT, PUBLISHED BOTH WAYS — HOW THE MARKET IS MEASURED. The same weekly regression of the</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" s="3" t="inlineStr"/>
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>stock's own returns is run against two different measures of its market, and the answer moves a long way</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>What it is not. It is not investment advice, a recommendation, or a price target. Values are model outputs</t>
+          <t>between them. Against the published index of the exchange the share is listed on — the index the method</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>shown as ranges and distributions.</t>
+          <t>asks for, and the primary reading — the beta is 1.103. Against an equal-weight composite of that same</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="3" t="inlineStr"/>
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>exchange's names, which gives its smallest listings the same say as its largest, the beta is</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>Sourcing note, up front. FY2023, FY2024 and FY2025 come from the company's own audited consolidated</t>
+          <t>0.705. The published index is weighted by size and is therefore dominated by the very group this</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>financial statements; the first quarter of 2026 comes from the reviewed interim statements; the fleet,</t>
+          <t>company belongs to; the composite is not. That single difference in construction, and nothing about the</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>rate and contract data come from the company's own investor presentations and earnings calls. Every input</t>
+          <t>company, moves the cost of equity and the cash-flow value materially. BOTH are carried through the model in</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>is listed with its value, source and date in the companion bibliography document.</t>
+          <t>full, side by side, on the Summary, Fundamental Valuation and DCF sheets. They are NOT averaged into one</t>
         </is>
       </c>
     </row>
     <row r="110">
-      <c r="A110" s="3" t="inlineStr"/>
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>number. The regression's own 90% confidence interval on the primary estimate runs 0.586 to 1.621, and</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>Currency. US dollar thousand unless stated — the company reports in US dollars. Per-share figures are in</t>
+          <t>those two bounds — not round numbers chosen by hand — are the betas used in the bear and bull cases, so the</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>dirhams at the fixed parity of 3.6725 dirhams to the dollar. Spot AED 6.16 (2026-08-07 close).</t>
+          <t>published range is the range the estimate itself supports.</t>
         </is>
       </c>
     </row>
     <row r="113">
-      <c r="A113" s="3" t="inlineStr">
-        <is>
-          <t>Sheets: READ FIRST · Summary · Fundamental Valuation · Assumptions · SOTP Bridge · Segments · Relative &amp;</t>
-        </is>
-      </c>
+      <c r="A113" s="3" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>Normalized · DCF · Income Statement · Balance Sheet · Cash Flow · Summary Financials · Monte Carlo ·</t>
+          <t>What it is not. It is not investment advice, a recommendation, or a price target. Values are model outputs</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
+        <is>
+          <t>shown as ranges and distributions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="3" t="inlineStr">
+        <is>
+          <t>Sourcing note, up front. FY2023, FY2024 and FY2025 come from the company's own audited consolidated</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>financial statements; the first quarter of 2026 comes from the reviewed interim statements; the fleet,</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="3" t="inlineStr">
+        <is>
+          <t>rate and contract data come from the company's own investor presentations and earnings calls. Every input</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>is listed with its value, source and date in the companion bibliography document.</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="3" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>Currency. US dollar thousand unless stated — the company reports in US dollars. Per-share figures are in</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="3" t="inlineStr">
+        <is>
+          <t>dirhams at the fixed parity of 3.6725 dirhams to the dollar. Spot AED 6.16 (2026-08-07 close).</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>Sheets: READ FIRST · Summary · Fundamental Valuation · Assumptions · SOTP Bridge · Segments · Relative &amp;</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="3" t="inlineStr">
+        <is>
+          <t>Normalized · DCF · Income Statement · Balance Sheet · Cash Flow · Summary Financials · Monte Carlo ·</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="3" t="inlineStr">
         <is>
           <t>Sensitivity · Per-Share &amp; Ratios · Peer &amp; Sector.</t>
         </is>
@@ -5497,64 +5570,64 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>1.085</t>
+          <t>1.103</t>
         </is>
       </c>
       <c r="B8" s="21" t="n">
-        <v>6.104211768824626</v>
+        <v>6.020153084134909</v>
       </c>
       <c r="C8" s="21" t="n">
-        <v>6.290365806735382</v>
+        <v>6.198777837752638</v>
       </c>
       <c r="D8" s="21" t="n">
-        <v>6.50557697172203</v>
+        <v>6.404817896532908</v>
       </c>
       <c r="E8" s="21" t="n">
-        <v>6.758173447014873</v>
+        <v>6.646025779733348</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>1.250</t>
+          <t>1.350</t>
         </is>
       </c>
       <c r="B9" s="21" t="n">
-        <v>5.400935220772635</v>
+        <v>5.031072269544037</v>
       </c>
       <c r="C9" s="21" t="n">
-        <v>5.528638734441224</v>
+        <v>5.132117653317763</v>
       </c>
       <c r="D9" s="21" t="n">
-        <v>5.673387508676271</v>
+        <v>5.245334010186813</v>
       </c>
       <c r="E9" s="21" t="n">
-        <v>5.839532255632811</v>
+        <v>5.373634668456338</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>1.412</t>
+          <t>1.621</t>
         </is>
       </c>
       <c r="B10" s="21" t="n">
-        <v>4.819724922415764</v>
+        <v>4.192019140583034</v>
       </c>
       <c r="C10" s="21" t="n">
-        <v>4.906776041409081</v>
+        <v>4.242712935566582</v>
       </c>
       <c r="D10" s="21" t="n">
-        <v>5.003609464167625</v>
+        <v>4.297604675716044</v>
       </c>
       <c r="E10" s="21" t="n">
-        <v>5.112479795523905</v>
+        <v>4.357554251269803</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>The beta rows are not evenly spaced round numbers. They span the two index constructions and the interval around the adopted one: 0.705 is the equal-weight composite of the exchange's own names, 1.085 is the adopted regression against the exchange's published index, and 1.412 is the top of that regression's own 90% confidence interval (its bottom, 0.758, sits just above the composite reading). The terminal growth column at 2.0% is the one the model runs on, so the cell where that column meets the 1.085 row is the published cash-flow value of AED 6.51 — every cell here is a complete re-run of the model discounted at the same three tranches of capital the valuation itself uses, equity, debt and the perpetual securities, so the grid is centred on the figure it brackets.</t>
+          <t>The beta rows are not evenly spaced round numbers. They span the two index constructions and the interval around the adopted one: 0.705 is the equal-weight composite of the exchange's own names, 1.103 is the adopted regression against the exchange's published index, and 1.621 is the top of that regression's own 90% confidence interval (its bottom, 0.586, sits below the composite reading, so the bull case is struck outside this grid). The terminal growth column at 2.0% is the one the model runs on, so the cell where that column meets the 1.103 row is the published cash-flow value of AED 6.40 — every cell here is a complete re-run of the model discounted at the same three tranches of capital the valuation itself uses, equity, debt and the perpetual securities, so the grid is centred on the figure it brackets.</t>
         </is>
       </c>
     </row>
@@ -5607,19 +5680,19 @@
         </is>
       </c>
       <c r="B14" s="21" t="n">
-        <v>5.466895404238599</v>
+        <v>5.380506785289913</v>
       </c>
       <c r="C14" s="21" t="n">
-        <v>5.986236187980316</v>
+        <v>5.892662340911411</v>
       </c>
       <c r="D14" s="21" t="n">
-        <v>6.50557697172203</v>
+        <v>6.404817896532908</v>
       </c>
       <c r="E14" s="21" t="n">
-        <v>7.024917755463745</v>
+        <v>6.916973452154407</v>
       </c>
       <c r="F14" s="21" t="n">
-        <v>7.544258539205458</v>
+        <v>7.429129007775901</v>
       </c>
     </row>
     <row r="15">
@@ -5636,7 +5709,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>This row and the one below it are re-runs of the whole model at the same 8.49% cost of capital the valuation uses, so the 1.00x cell reproduces the published AED 6.51 exactly and the swing across the row is a clean read of what that single driver is worth.</t>
+          <t>This row and the one below it are re-runs of the whole model at the same 8.56% cost of capital the valuation uses, so the 1.00x cell reproduces the published AED 6.40 exactly and the swing across the row is a clean read of what that single driver is worth.</t>
         </is>
       </c>
     </row>
@@ -5684,16 +5757,16 @@
         </is>
       </c>
       <c r="B19" s="21" t="n">
-        <v>6.914940440302763</v>
+        <v>6.81087218594573</v>
       </c>
       <c r="C19" s="21" t="n">
-        <v>6.50557697172203</v>
+        <v>6.404817896532908</v>
       </c>
       <c r="D19" s="21" t="n">
-        <v>6.096213503141294</v>
+        <v>5.998763607120084</v>
       </c>
       <c r="E19" s="21" t="n">
-        <v>5.686850034560557</v>
+        <v>5.592709317707262</v>
       </c>
     </row>
     <row r="20">
@@ -5746,13 +5819,13 @@
         </is>
       </c>
       <c r="B24" s="21" t="n">
-        <v>6.415224723153202</v>
+        <v>6.315163657148892</v>
       </c>
       <c r="C24" s="21" t="n">
-        <v>5.963130365206823</v>
+        <v>5.868212089093989</v>
       </c>
       <c r="D24" s="21" t="n">
-        <v>5.284988828287254</v>
+        <v>5.197784737011633</v>
       </c>
     </row>
     <row r="25">
@@ -7981,11 +8054,11 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>beta 1.412 — the TOP of the regression's own 90% confidence interval, not a round number picked by hand — with the rate anchor at 0.85x and capital expenditure at 1.10x. A whole-model re-run</t>
+          <t>beta 1.621 — the TOP of the regression's own 90% confidence interval, not a round number picked by hand — with the rate anchor at 0.85x and capital expenditure at 1.10x. A whole-model re-run</t>
         </is>
       </c>
       <c r="C6" s="21" t="n">
-        <v>4.025007328525061</v>
+        <v>3.417404968021705</v>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
@@ -7996,11 +8069,11 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>beta 0.758 — the BOTTOM of the same interval — with the rate anchor at 1.15x and capital expenditure at 0.95x. Taking both bounds from the interval means the published range is the range the estimate itself supports. A whole-model re-run</t>
+          <t>beta 0.586 — the BOTTOM of the same interval — with the rate anchor at 1.15x and capital expenditure at 0.95x. Taking both bounds from the interval means the published range is the range the estimate itself supports. A whole-model re-run</t>
         </is>
       </c>
       <c r="C7" s="21" t="n">
-        <v>10.13215941638862</v>
+        <v>12.2389432347382</v>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
@@ -8080,7 +8153,7 @@
       </c>
       <c r="B15" s="20" t="inlineStr">
         <is>
-          <t>161 weekly observations, R-squared 15.8%, standard error 0.199, 90% confidence interval 0.758 to 1.412 — the usability gate is passed, and this is the index the method asks for</t>
+          <t>159 weekly observations, R-squared 18.1%, standard error 0.315, 90% confidence interval 0.586 to 1.621 — the usability gate is passed, and this is the index the method asks for</t>
         </is>
       </c>
       <c r="C15" s="23">
@@ -8342,13 +8415,13 @@
         </is>
       </c>
       <c r="C32" s="21" t="n">
-        <v>6.302103806955713</v>
+        <v>6.226950849542018</v>
       </c>
       <c r="D32" s="21" t="n">
-        <v>4.612173662625463</v>
+        <v>4.183627650976118</v>
       </c>
       <c r="E32" s="21" t="n">
-        <v>8.85643410508878</v>
+        <v>10.54299487474104</v>
       </c>
     </row>
     <row r="33">
@@ -8363,13 +8436,13 @@
         </is>
       </c>
       <c r="C33" s="21" t="n">
-        <v>4.892938708214075</v>
+        <v>4.798904529252498</v>
       </c>
       <c r="D33" s="21" t="n">
-        <v>3.481417824283891</v>
+        <v>3.432639967125382</v>
       </c>
       <c r="E33" s="21" t="n">
-        <v>5.996520587194937</v>
+        <v>5.866633504326449</v>
       </c>
     </row>
     <row r="34">
@@ -8536,7 +8609,7 @@
         </is>
       </c>
       <c r="C14" s="29" t="n">
-        <v>1.085</v>
+        <v>1.1032</v>
       </c>
     </row>
     <row r="15">
@@ -8556,7 +8629,7 @@
         </is>
       </c>
       <c r="C16" s="29" t="n">
-        <v>0.758</v>
+        <v>0.5855</v>
       </c>
     </row>
     <row r="17">
@@ -8566,17 +8639,17 @@
         </is>
       </c>
       <c r="C17" s="29" t="n">
-        <v>1.412</v>
+        <v>1.621</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>Beta — lead-lag sum beta from the same series, one lead and two lags</t>
+          <t>Beta — the measured slope shrunk toward the market: two-thirds of it plus one-third of 1.0</t>
         </is>
       </c>
       <c r="C18" s="29" t="n">
-        <v>1.164</v>
+        <v>1.0688</v>
       </c>
     </row>
     <row r="19">
@@ -19449,7 +19522,7 @@
     <row r="125">
       <c r="A125" s="6" t="inlineStr">
         <is>
-          <t>Beta — lead-lag sum beta, one lead and two lags</t>
+          <t>Beta — the measured slope shrunk toward the market, two-thirds of it plus one-third of 1.0</t>
         </is>
       </c>
       <c r="C125" s="23">
@@ -19460,7 +19533,7 @@
     <row r="126">
       <c r="A126" s="6" t="inlineStr">
         <is>
-          <t>Cost of equity on the lead-lag sum beta</t>
+          <t>Cost of equity on the slope shrunk toward the market</t>
         </is>
       </c>
       <c r="C126" s="50">

</xml_diff>